<commit_message>
überarbeitete Formeln zu CO2-Berechnung
</commit_message>
<xml_diff>
--- a/DP_ACBAY/Backend/data/emissionen_nach_typ.xlsx
+++ b/DP_ACBAY/Backend/data/emissionen_nach_typ.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Pendelweg" sheetId="1" state="visible" r:id="rId1"/>
@@ -405,14 +405,10 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-      <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -435,9 +431,6 @@
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
       <protection hidden="0" locked="1"/>
@@ -451,8 +444,6 @@
       <alignment readingOrder="0" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -977,111 +968,111 @@
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>235</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" ht="15">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>234</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>188</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="30">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>163</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" ht="15">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>63</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>52</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" ht="30">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>203</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" ht="30">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>210</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E9" t="s">
@@ -1089,16 +1080,16 @@
       </c>
     </row>
     <row r="10" ht="15">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>100</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E10" t="s">
@@ -1106,16 +1097,16 @@
       </c>
     </row>
     <row r="11" ht="15">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>55</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E11" t="s">
@@ -1123,30 +1114,30 @@
       </c>
     </row>
     <row r="12" ht="15">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <v>25</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" ht="45">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <v>10</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E13" t="s">
@@ -1154,116 +1145,116 @@
       </c>
     </row>
     <row r="14" ht="15">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <v>20</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" ht="15">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="2">
         <v>20</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F15" s="4"/>
+      <c r="F15" s="3"/>
     </row>
     <row r="16" ht="30">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="2">
         <v>5</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" ht="30">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
     </row>
     <row r="18" ht="30">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
     </row>
     <row r="19" ht="30">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
     </row>
     <row r="20" ht="30">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20" s="2">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
     </row>
     <row r="21" ht="30">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" s="2">
         <f>1/10</f>
         <v>0.10000000000000001</v>
       </c>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
     </row>
     <row r="22" ht="30">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22" s="2">
         <f>1/30</f>
         <v>3.3333333333333333e-002</v>
       </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
     </row>
     <row r="23" ht="30">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23" s="2">
         <v>0</v>
       </c>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
     </row>
     <row r="24" ht="30"/>
     <row r="25" ht="15"/>
@@ -1273,7 +1264,7 @@
       </c>
     </row>
     <row r="27" ht="15">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B27">
@@ -1287,7 +1278,7 @@
       </c>
     </row>
     <row r="28" ht="15">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="4" t="s">
         <v>40</v>
       </c>
       <c r="B28">
@@ -1296,12 +1287,12 @@
       <c r="C28" t="s">
         <v>38</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="29" ht="45">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="4" t="s">
         <v>41</v>
       </c>
       <c r="B29">
@@ -1310,7 +1301,7 @@
       <c r="C29" t="s">
         <v>38</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="5" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1324,7 +1315,7 @@
       <c r="C30" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="5" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1338,7 +1329,7 @@
       <c r="C31" t="s">
         <v>38</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="5" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1352,7 +1343,7 @@
       <c r="C32" t="s">
         <v>38</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="5" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1367,7 +1358,7 @@
       <c r="A36">
         <v>0</v>
       </c>
-      <c r="B36" s="7">
+      <c r="B36" s="6">
         <v>0</v>
       </c>
       <c r="C36" t="s">
@@ -1381,13 +1372,13 @@
       <c r="A37">
         <v>1</v>
       </c>
-      <c r="B37" s="7">
+      <c r="B37" s="6">
         <v>1</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="5" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1395,13 +1386,13 @@
       <c r="A38">
         <v>2</v>
       </c>
-      <c r="B38" s="7">
+      <c r="B38" s="6">
         <v>2</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="5" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1409,13 +1400,13 @@
       <c r="A39">
         <v>3</v>
       </c>
-      <c r="B39" s="7">
+      <c r="B39" s="6">
         <v>3</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="5" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1423,13 +1414,13 @@
       <c r="A40">
         <v>4</v>
       </c>
-      <c r="B40" s="7">
+      <c r="B40" s="6">
         <v>4</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D40" s="5" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1437,13 +1428,13 @@
       <c r="A41">
         <v>5</v>
       </c>
-      <c r="B41" s="7">
+      <c r="B41" s="6">
         <v>5</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D41" s="5" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1451,26 +1442,26 @@
       <c r="A45" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
     </row>
     <row r="47" ht="14.25">
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
     </row>
     <row r="48" ht="14.25">
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1495,30 +1486,30 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>345</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>54</v>
       </c>
       <c r="E2" t="s">
@@ -1526,100 +1517,100 @@
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>225</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>313</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>26</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>25</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>172</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="8" ht="14.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>42</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="9">
         <v>138</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E9" t="s">
@@ -1627,64 +1618,64 @@
       </c>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="6">
         <v>25</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="11" ht="14.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="10">
         <v>209</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="15" ht="14.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>18000</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>74</v>
       </c>
       <c r="E15" t="s">
@@ -1692,30 +1683,30 @@
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="9">
         <v>1000</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="9" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="9">
         <v>130</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="9" t="s">
         <v>80</v>
       </c>
       <c r="E17" t="s">
@@ -1728,26 +1719,30 @@
       </c>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14" t="s">
+      <c r="B20" s="12">
+        <v>6912</v>
+      </c>
+      <c r="C20" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="12" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14" t="s">
+      <c r="B21" s="12">
+        <v>1741</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="14"/>
+      <c r="D21" s="12"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -1782,17 +1777,17 @@
       </c>
     </row>
     <row r="2" ht="14">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="3">
-        <f>B16*B22*2</f>
+      <c r="B2" s="2">
+        <f t="shared" ref="B2:B4" si="0">B16*B22*2</f>
         <v>225000</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="13" t="s">
         <v>89</v>
       </c>
       <c r="F2" t="s">
@@ -1800,32 +1795,32 @@
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="3">
-        <f>B17*B23*2</f>
+      <c r="B3" s="2">
+        <f t="shared" si="0"/>
         <v>750000</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="3">
-        <f>B18*B24*2</f>
+      <c r="B4" s="2">
+        <f t="shared" si="0"/>
         <v>1500000</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1835,7 +1830,7 @@
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="16">
+      <c r="A9" s="4">
         <v>0</v>
       </c>
       <c r="B9">
@@ -1843,7 +1838,7 @@
       </c>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="4" t="s">
         <v>94</v>
       </c>
       <c r="B10">
@@ -1851,7 +1846,7 @@
       </c>
     </row>
     <row r="11" ht="14.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="4" t="s">
         <v>95</v>
       </c>
       <c r="B11">
@@ -1859,7 +1854,7 @@
       </c>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="4" t="s">
         <v>96</v>
       </c>
       <c r="B12">
@@ -1872,10 +1867,10 @@
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="12">
         <v>150</v>
       </c>
       <c r="C16" t="s">
@@ -1886,10 +1881,10 @@
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="9">
         <v>150</v>
       </c>
       <c r="C17" t="s">
@@ -1900,10 +1895,10 @@
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>150</v>
       </c>
       <c r="C18" t="s">
@@ -1970,7 +1965,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" ht="15">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
änderungen backend und datenbank
</commit_message>
<xml_diff>
--- a/DP_ACBAY/Backend/data/emissionen_nach_typ.xlsx
+++ b/DP_ACBAY/Backend/data/emissionen_nach_typ.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Pendelweg" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
   <si>
     <t xml:space="preserve">Mobilitätsart (2)</t>
   </si>
@@ -342,14 +342,104 @@
     <t xml:space="preserve">Langstrecke &gt;3500km</t>
   </si>
   <si>
-    <t xml:space="preserve">*vorläufig weggelassen</t>
+    <t>Kategorie</t>
+  </si>
+  <si>
+    <t>Basiswert_t_CO2e</t>
+  </si>
+  <si>
+    <t>Max_Reduktion_t_CO2e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesamtbasis (Ernährung + Konsumgüter + Alltagsmobilität)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t CO2e/Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC Consumer Footprint + Eurostat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durchschnittswerge ergänzen:</t>
+  </si>
+  <si>
+    <t>Ernährung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC Consumer Footprint</t>
+  </si>
+  <si>
+    <t>Konsumgüter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alltagsmobilität (ohne Pendeln)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC + Eurostat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAsierend auf angaben - Wertänderung (+/-)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nachhaltige Kleidung – immer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC Anteil Textilien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nachhaltige Kleidung – manchmal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regionaler Einkauf – oft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC Ernährung Transportanteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regionaler Einkauf – manchmal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verzicht auf Onlinekauf – oft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC Konsumgüter Logistikanteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verzicht auf Onlinekauf – manchmal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umweltfreundlicher Transport beim Einkauf – Ja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC Mobilitätsanteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umweltfreundlicher Transport beim Einkauf – Manchmal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energiesparende Geräte – alle (Herstellung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JRC Geräteanteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smarte Geräte – Ja (Herstellung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feuerwerk &gt;1/Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCA Literatur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feuerwerk 1/Jahr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -362,6 +452,17 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color indexed="64"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.000000"/>
+      <color indexed="64"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -405,7 +506,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -442,6 +543,25 @@
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -1968,8 +2088,327 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" ht="15">
-      <c r="A1" t="s">
+      <c r="A1" s="14" t="s">
         <v>107</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B2" s="16">
+        <v>5.5999999999999996</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="A3" s="14"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="15"/>
+    </row>
+    <row r="4" ht="14.25">
+      <c r="A4" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15"/>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" s="16">
+        <v>1.7</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="16">
+        <v>1.7</v>
+      </c>
+      <c r="C7" s="17"/>
+      <c r="D7" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" s="14"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="15"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="15"/>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="16">
+        <v>-0.20000000000000001</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="A11" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B11" s="17"/>
+      <c r="C11" s="16">
+        <v>-0.10000000000000001</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="15"/>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="A13" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="16">
+        <v>-0.12</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="17"/>
+      <c r="C14" s="16">
+        <v>-5.9999999999999998e-002</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="14"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="16">
+        <v>-0.14999999999999999</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="16">
+        <v>-7.0000000000000007e-002</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" s="14"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="15"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="B19" s="17"/>
+      <c r="C19" s="16">
+        <v>-0.20999999999999999</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="16">
+        <v>-0.10000000000000001</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" s="14"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="15"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="16">
+        <v>-8.9999999999999997e-002</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="A23" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B23" s="17"/>
+      <c r="C23" s="16">
+        <v>-5.0000000000000003e-002</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" s="14"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="16">
+        <v>1.e-002</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="16">
+        <v>5.0000000000000001e-003</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>